<commit_message>
User feedback stuffs (#3)
* User feedback stuffs

* không gọp tổng sl trong chi tiết đơn hàng

* không group chi tiết khi in

* UI bán hàng

* bugfixes

* remove ngx-print
</commit_message>
<xml_diff>
--- a/API/Resources/Template/Report/Download.xlsx
+++ b/API/Resources/Template/Report/Download.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABAC1639-CB50-4D4B-AC99-E304FADCCCBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,12 +15,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
   <si>
     <t>Tên Sản Phẩm</t>
   </si>
@@ -97,12 +101,18 @@
   </si>
   <si>
     <t>&amp;=result.DoanhThu</t>
+  </si>
+  <si>
+    <t>Mã Sản Phẩm</t>
+  </si>
+  <si>
+    <t>&amp;=result.MaSP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -142,7 +152,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -174,11 +184,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -204,6 +240,9 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -214,6 +253,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -500,151 +545,161 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" style="3" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" style="3" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" style="3" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" style="2" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" style="3" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" style="3" customWidth="1"/>
+    <col min="11" max="11" width="20.7109375" style="2" customWidth="1"/>
+    <col min="12" max="12" width="20.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10"/>
+      <c r="G3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="10"/>
+      <c r="I3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="10"/>
+      <c r="K3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="9"/>
+      <c r="L3" s="10"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="4" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="10"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="L4" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="K5" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="8"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
@@ -652,19 +707,21 @@
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>